<commit_message>
Code is being modularised
</commit_message>
<xml_diff>
--- a/reports/NBA_Attainment_Report.xlsx
+++ b/reports/NBA_Attainment_Report.xlsx
@@ -664,17 +664,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cxzds</t>
+          <t>asd</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>dfsdf</t>
+          <t>asd</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>sdf</t>
+          <t>asd</t>
         </is>
       </c>
     </row>

</xml_diff>